<commit_message>
end: rendre les nombres de véhicules optionnels
fixes #434

Les validations sur le nombre de véhicules à la section fin sont
maintenant optionnelles. Puisque la validation sur le nombre dépend du
carNumber, qui devrait avoir été validé selon le nombre de membres du
ménage, seule la validation comparée est nécessaires ici, ce qui enlève
le required qui vient avec les validations de véhicules.
</commit_message>
<xml_diff>
--- a/survey/references/OD_mtl_2026.xlsx
+++ b/survey/references/OD_mtl_2026.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Widgets" sheetId="1" state="visible" r:id="rId3"/>
@@ -3636,7 +3636,7 @@
     <t xml:space="preserve">householdHasCars</t>
   </si>
   <si>
-    <t xml:space="preserve">householdHybridCarCountCustomValidation</t>
+    <t xml:space="preserve">householdHybridCarCountOrOptionalCustomValidation</t>
   </si>
   <si>
     <t xml:space="preserve">householdElectricCarNumber</t>
@@ -3653,7 +3653,7 @@
 __Optional__</t>
   </si>
   <si>
-    <t xml:space="preserve">householdElectricCarCountCustomValidation</t>
+    <t xml:space="preserve">householdElectricCarCountOrOptionalCustomValidation</t>
   </si>
   <si>
     <t xml:space="preserve">householdIncome</t>
@@ -13099,6 +13099,7 @@
         <v>360</v>
       </c>
       <c r="C79" s="1" t="b">
+        <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
       <c r="D79" s="1" t="s">

</xml_diff>